<commit_message>
Updated content of the 'references/Notes.xlsx'
</commit_message>
<xml_diff>
--- a/references/Notes.xlsx
+++ b/references/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Bank System Related Stuffs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31975EE9-A7EC-4729-AAF8-A8A7374FF9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B64C76B9-EE2B-4740-962C-0FAB6D4BCC91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="54">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -859,6 +859,9 @@
       <c r="G14" s="5" t="s">
         <v>40</v>
       </c>
+      <c r="I14" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -867,6 +870,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1010,15 +1022,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -1026,6 +1029,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1039,14 +1050,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Modify the content of the DBML file and the Notes.xlsx file. Added new files
</commit_message>
<xml_diff>
--- a/references/Notes.xlsx
+++ b/references/Notes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Bank System Related Stuffs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B64C76B9-EE2B-4740-962C-0FAB6D4BCC91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBDFF19B-C087-4F71-AE57-59C2D300A282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="57">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -144,9 +144,6 @@
     <t>Binigay na ni maam Joana thru hardcopy</t>
   </si>
   <si>
-    <t>Update mo si Maam Joana kung kailan pwede makuha thru email</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -196,6 +193,18 @@
   </si>
   <si>
     <t>Sir Nico kaso nakaleave, nasa gilid siya, pwede naman daw ako gumawa muna ng initial ERD ko for that. May binigay na context sa akin si Sir Jap, naka time-based daw yung pag-track ng progress percentage ng mga master development plan and dapat tinatrack ko siya per barangay and not total barangay. Every 3 years dapat tinatrack ko yung progress percentage. Dapat din may 3 types of plans na sinasubmit bawat plan (Initial, Revised, Approved). Kung sakop pa ng range niya yung Date Range sa sinubmit na Plan, dapat updated yun</t>
+  </si>
+  <si>
+    <t>Hintayin or update si Ma'am Joana kung kailan makukuha yung raw data for this indicator</t>
+  </si>
+  <si>
+    <t>same sa nasa taas</t>
+  </si>
+  <si>
+    <t>running average. Tanong nalang uli kay sir Jap</t>
+  </si>
+  <si>
+    <t>Kay Sir Jap lang ako nagtanong kaya binigyan ako ng column. Tanong mo nalang saan galing yung data na sinend niya sa akin. annually, may target pct per 3 years, pero index crime lang siya.</t>
   </si>
 </sst>
 </file>
@@ -609,7 +618,7 @@
         <v>33</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -638,7 +647,7 @@
         <v>34</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -661,13 +670,13 @@
         <v>30</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="I3" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="144" x14ac:dyDescent="0.3">
@@ -690,13 +699,13 @@
         <v>30</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="67.2" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -720,13 +729,13 @@
         <v>30</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>35</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -749,47 +758,50 @@
         <v>30</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>25</v>
@@ -801,21 +813,24 @@
         <v>25</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>25</v>
@@ -827,25 +842,28 @@
         <v>25</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>55</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>25</v>
@@ -854,13 +872,13 @@
         <v>25</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -870,15 +888,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1022,6 +1031,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -1029,14 +1047,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1050,6 +1060,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Added notes to the content of the Notes.xlsx
</commit_message>
<xml_diff>
--- a/references/Notes.xlsx
+++ b/references/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBDFF19B-C087-4F71-AE57-59C2D300A282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEEDF83-26FF-488D-BB1D-2E22A3D9D27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -204,7 +204,20 @@
     <t>running average. Tanong nalang uli kay sir Jap</t>
   </si>
   <si>
-    <t>Kay Sir Jap lang ako nagtanong kaya binigyan ako ng column. Tanong mo nalang saan galing yung data na sinend niya sa akin. annually, may target pct per 3 years, pero index crime lang siya.</t>
+    <r>
+      <t xml:space="preserve">Kay Sir Jap lang ako nagtanong kaya binigyan ako ng column. Tanong mo nalang saan galing yung data na sinend niya sa akin. annually, may target pct per 3 years, pero index crime lang siya. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NOTES: Importante lang na mabilang yung crime rate to get the reduction percentage so get the necessary data</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -767,7 +780,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
@@ -1032,18 +1045,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1065,14 +1078,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1086,4 +1091,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the status column from the Notes.xlsx
</commit_message>
<xml_diff>
--- a/references/Notes.xlsx
+++ b/references/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEEDF83-26FF-488D-BB1D-2E22A3D9D27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21556757-2B6E-4F79-8084-56CCED34597D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -806,7 +806,7 @@
         <v>56</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -901,6 +901,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1044,35 +1059,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1094,9 +1084,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the status of the Note excel file
</commit_message>
<xml_diff>
--- a/references/Notes.xlsx
+++ b/references/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21556757-2B6E-4F79-8084-56CCED34597D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C52BEEE8-88E2-4724-851B-2AEBCB98B67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -198,9 +198,6 @@
     <t>Hintayin or update si Ma'am Joana kung kailan makukuha yung raw data for this indicator</t>
   </si>
   <si>
-    <t>same sa nasa taas</t>
-  </si>
-  <si>
     <t>running average. Tanong nalang uli kay sir Jap</t>
   </si>
   <si>
@@ -218,6 +215,9 @@
       </rPr>
       <t>NOTES: Importante lang na mabilang yung crime rate to get the reduction percentage so get the necessary data</t>
     </r>
+  </si>
+  <si>
+    <t>same sa nasa taas ang pagkakaiba yung data sa pagmemeasure nila. PNP - Barangay, MBDA - Latitude/Longitude</t>
   </si>
 </sst>
 </file>
@@ -803,7 +803,7 @@
         <v>39</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>37</v>
@@ -832,10 +832,10 @@
         <v>39</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -861,7 +861,7 @@
         <v>39</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>38</v>
@@ -901,18 +901,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1060,14 +1060,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1079,6 +1071,14 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Modify the status inside the 'Notes.xlsx'
</commit_message>
<xml_diff>
--- a/references/Notes.xlsx
+++ b/references/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C52BEEE8-88E2-4724-851B-2AEBCB98B67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1353A107-DC00-4D0C-90AF-7B4E7248E8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -907,15 +907,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1059,6 +1050,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
@@ -1076,14 +1076,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1099,4 +1091,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the status inside the content of the `references\Notes.xlsx`
</commit_message>
<xml_diff>
--- a/references/Notes.xlsx
+++ b/references/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1353A107-DC00-4D0C-90AF-7B4E7248E8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16622ABB-D531-48C7-9626-86353FDA67A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="58">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -218,6 +218,9 @@
   </si>
   <si>
     <t>same sa nasa taas ang pagkakaiba yung data sa pagmemeasure nila. PNP - Barangay, MBDA - Latitude/Longitude</t>
+  </si>
+  <si>
+    <t>ONGOING</t>
   </si>
 </sst>
 </file>
@@ -864,7 +867,7 @@
         <v>54</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -901,9 +904,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1051,26 +1057,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1094,9 +1089,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refact: Content of the status of the `references\Notes.xlsx`
</commit_message>
<xml_diff>
--- a/references/Notes.xlsx
+++ b/references/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16622ABB-D531-48C7-9626-86353FDA67A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4CC5D51-5974-47F0-8F51-4AF394BB52F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -198,9 +198,6 @@
     <t>Hintayin or update si Ma'am Joana kung kailan makukuha yung raw data for this indicator</t>
   </si>
   <si>
-    <t>running average. Tanong nalang uli kay sir Jap</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Kay Sir Jap lang ako nagtanong kaya binigyan ako ng column. Tanong mo nalang saan galing yung data na sinend niya sa akin. annually, may target pct per 3 years, pero index crime lang siya. </t>
     </r>
@@ -221,6 +218,9 @@
   </si>
   <si>
     <t>ONGOING</t>
+  </si>
+  <si>
+    <t>running average. Injury count total in any injury types and severities</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
         <v>39</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>37</v>
@@ -835,7 +835,7 @@
         <v>39</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>37</v>
@@ -864,10 +864,10 @@
         <v>39</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -913,6 +913,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1056,12 +1062,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
@@ -1071,6 +1071,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1086,20 +1102,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>